<commit_message>
Periodic update to ensure github version
</commit_message>
<xml_diff>
--- a/data/defaultSpread.xlsx
+++ b/data/defaultSpread.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jhess/Documents/Investing/Damodaran Reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9999B5-1370-5B4A-BA03-13E06A5273EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565CA240-889F-A647-BC29-3BCE785C40CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32140" yWindow="560" windowWidth="28040" windowHeight="16940" xr2:uid="{09585497-DD20-934D-85B3-5D578C09CEB9}"/>
+    <workbookView xWindow="40960" yWindow="1500" windowWidth="28040" windowHeight="16940" xr2:uid="{09585497-DD20-934D-85B3-5D578C09CEB9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -153,9 +153,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -193,7 +193,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -299,7 +299,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -441,7 +441,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -452,7 +452,8 @@
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10.83203125" style="3"/>
+    <col min="1" max="1" width="10.83203125" style="3"/>
+    <col min="2" max="2" width="12.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" style="1"/>
     <col min="4" max="4" width="10.83203125" style="2"/>
   </cols>
@@ -672,7 +673,7 @@
         <v>12.5</v>
       </c>
       <c r="B16" s="3">
-        <v>100000</v>
+        <v>100000000</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>16</v>

</xml_diff>